<commit_message>
feat: add 9th WAS monthly employee 94318 Suphamongkol Phiwkhom and update counts
</commit_message>
<xml_diff>
--- a/scans_was/WAS_รายเดือน.xlsx
+++ b/scans_was/WAS_รายเดือน.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://goodyearcorp-my.sharepoint.com/personal/nichakamon_kaewkeadmee_goodyear_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aa11909\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D964A522-2A8B-4928-93FD-243F16562838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9898EF57-4DCE-4836-A91D-5CD068945CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9F4C0C6D-8ABB-40A4-B8E1-6FE0F2124004}"/>
   </bookViews>
@@ -17,7 +17,6 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
-    <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
     <definedName name="\0">#REF!</definedName>
@@ -13569,7 +13568,7 @@
     <definedName name="sls_ytd_pyr">#REF!</definedName>
     <definedName name="slss">#REF!</definedName>
     <definedName name="SMO">#REF!</definedName>
-    <definedName name="Social_Rate">[2]ACTIVE!$AF$7</definedName>
+    <definedName name="Social_Rate">[1]ACTIVE!$AF$7</definedName>
     <definedName name="soe">#REF!</definedName>
     <definedName name="SOH">#REF!</definedName>
     <definedName name="soldirection">OFFSET(#REF!,0,0,COUNTA(#REF!))</definedName>
@@ -14547,7 +14546,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="45">
   <si>
     <t>World Asia Solution Co.,Ltd.</t>
   </si>
@@ -14670,6 +14669,18 @@
   </si>
   <si>
     <t>Quality</t>
+  </si>
+  <si>
+    <t>Suphamongkol Phiwkhom</t>
+  </si>
+  <si>
+    <t>ศุภมงคล ผิวขม</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RE </t>
+  </si>
+  <si>
+    <t>BCB</t>
   </si>
 </sst>
 </file>
@@ -14895,40 +14906,6 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="AOP Sep'26"/>
-      <sheetName val="Vacancies"/>
-      <sheetName val="Data employee"/>
-      <sheetName val="Hourly+Salary (เข้า-ออก)"/>
-      <sheetName val="Hourly"/>
-      <sheetName val="Vacancies and Training"/>
-      <sheetName val="Salary"/>
-      <sheetName val="Service contrace"/>
-      <sheetName val="Service contrace hourly"/>
-      <sheetName val="Sheet1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -15260,24 +15237,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6782B530-3559-450C-A78B-527ACC167DB6}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="20"/>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="20.399999999999999"/>
   <cols>
-    <col min="1" max="1" width="4.81640625" style="23" customWidth="1"/>
-    <col min="2" max="2" width="14.453125" style="23" customWidth="1"/>
-    <col min="3" max="3" width="29.08984375" style="24" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.77734375" style="23" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="23" customWidth="1"/>
+    <col min="3" max="3" width="29.109375" style="24" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" style="24" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.1796875" style="24" customWidth="1"/>
+    <col min="5" max="5" width="29.21875" style="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.21875" style="24" customWidth="1"/>
     <col min="7" max="7" width="9" style="23" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.90625" style="24" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.54296875" style="24" customWidth="1"/>
-    <col min="10" max="10" width="21.36328125" style="24" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.08984375" style="26" customWidth="1"/>
-    <col min="12" max="16384" width="9.1796875" style="26"/>
+    <col min="8" max="8" width="9.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" style="24" customWidth="1"/>
+    <col min="10" max="10" width="21.33203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.109375" style="26" customWidth="1"/>
+    <col min="12" max="16384" width="9.21875" style="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="8" customFormat="1" ht="29">
+    <row r="1" spans="1:10" s="8" customFormat="1" ht="28.8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -15291,7 +15268,7 @@
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
     </row>
-    <row r="2" spans="1:10" s="8" customFormat="1" ht="29">
+    <row r="2" spans="1:10" s="8" customFormat="1" ht="28.8">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -15305,7 +15282,7 @@
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
     </row>
-    <row r="3" spans="1:10" s="15" customFormat="1" ht="23">
+    <row r="3" spans="1:10" s="15" customFormat="1" ht="23.4">
       <c r="A3" s="13" t="s">
         <v>2</v>
       </c>
@@ -15337,7 +15314,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="21" customFormat="1" ht="23">
+    <row r="4" spans="1:10" s="21" customFormat="1" ht="23.4">
       <c r="A4" s="16">
         <f>1</f>
         <v>1</v>
@@ -15370,7 +15347,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="21" customFormat="1" ht="23">
+    <row r="5" spans="1:10" s="21" customFormat="1" ht="23.4">
       <c r="A5" s="16">
         <f t="shared" ref="A5:A11" si="0">A4+1</f>
         <v>2</v>
@@ -15403,7 +15380,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="21" customFormat="1" ht="23">
+    <row r="6" spans="1:10" s="21" customFormat="1" ht="23.4">
       <c r="A6" s="16">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -15436,7 +15413,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" s="21" customFormat="1" ht="23">
+    <row r="7" spans="1:10" s="21" customFormat="1" ht="23.4">
       <c r="A7" s="16">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -15469,7 +15446,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:10" s="21" customFormat="1" ht="23">
+    <row r="8" spans="1:10" s="21" customFormat="1" ht="23.4">
       <c r="A8" s="16">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -15502,7 +15479,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="21" customFormat="1" ht="23">
+    <row r="9" spans="1:10" s="21" customFormat="1" ht="23.4">
       <c r="A9" s="16">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -15535,7 +15512,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:10" s="21" customFormat="1" ht="23">
+    <row r="10" spans="1:10" s="21" customFormat="1" ht="23.4">
       <c r="A10" s="16">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -15568,7 +15545,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:10" s="21" customFormat="1" ht="23">
+    <row r="11" spans="1:10" s="21" customFormat="1" ht="23.4">
       <c r="A11" s="16">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -15601,6 +15578,36 @@
         <v>18</v>
       </c>
     </row>
+    <row r="12" spans="1:10" ht="23.4">
+      <c r="A12" s="16">
+        <v>9</v>
+      </c>
+      <c r="B12" s="20">
+        <v>94318</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" s="20">
+        <v>5120</v>
+      </c>
+      <c r="H12" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12" s="22"/>
+      <c r="J12" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>